<commit_message>
New demo files, only demo complete for now.
</commit_message>
<xml_diff>
--- a/demo/demo4-complete/output/post-method-series.xlsx
+++ b/demo/demo4-complete/output/post-method-series.xlsx
@@ -555,13 +555,13 @@
         <v>2015</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>9129.500547667343</v>
+        <v>9288.188185990821</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>9975.274312943264</v>
+        <v>10315.40580673759</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>1.092641843971631</v>
+        <v>1.110593971631206</v>
       </c>
     </row>
     <row r="4">
@@ -569,13 +569,13 @@
         <v>2016</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>12367.60284069755</v>
+        <v>12367.80845969673</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>13768.70739674955</v>
+        <v>13961.13873873874</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>1.113288288288288</v>
+        <v>1.128828828828829</v>
       </c>
     </row>
     <row r="5">
@@ -583,13 +583,13 @@
         <v>2017</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>7590.37827067754</v>
+        <v>7906.449556093624</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>9031.349803216955</v>
+        <v>9492.336240310078</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1.189841860465116</v>
+        <v>1.200581395348837</v>
       </c>
     </row>
     <row r="6">
@@ -597,13 +597,13 @@
         <v>2018</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>12192.26847879501</v>
+        <v>12220.54106570513</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>16292.8457012075</v>
+        <v>16346.44721329046</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1.336326027395498</v>
+        <v>1.337620578778135</v>
       </c>
     </row>
     <row r="7">
@@ -611,13 +611,13 @@
         <v>2019</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>9452.312274849644</v>
+        <v>9685.77439516129</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>13124.46684429074</v>
+        <v>13419.3969273743</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>1.388492726717443</v>
+        <v>1.385474860335196</v>
       </c>
     </row>
     <row r="8">
@@ -625,13 +625,13 @@
         <v>2020</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>8731.988870919324</v>
+        <v>9026.448533872599</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>13367.35091242506</v>
+        <v>13670.99173047473</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1.530848367998174</v>
+        <v>1.514548238897397</v>
       </c>
     </row>
     <row r="9">
@@ -639,13 +639,13 @@
         <v>2021</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>14662.03317115164</v>
+        <v>14429.98176718093</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>24133.73918177336</v>
+        <v>23322.55148963731</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1.646002222205978</v>
+        <v>1.616256476683938</v>
       </c>
     </row>
     <row r="10">
@@ -653,13 +653,13 @@
         <v>2022</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>9402.372271680102</v>
+        <v>9584.186523239294</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>13400.46162007459</v>
+        <v>13616.28806228374</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1.425221341260515</v>
+        <v>1.420703575547866</v>
       </c>
     </row>
     <row r="11">
@@ -667,13 +667,13 @@
         <v>2023</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>10488.92748269362</v>
+        <v>10454.63747810858</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>15263.78647048895</v>
+        <v>15360.81826954004</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>1.455228525096936</v>
+        <v>1.469282727565133</v>
       </c>
     </row>
     <row r="12">
@@ -681,13 +681,13 @@
         <v>2024</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>11870.65479375138</v>
+        <v>12108.97857689365</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>18275.77580410895</v>
+        <v>19966.06602186711</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1.539576048806438</v>
+        <v>1.648864592094197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Better formatting on complete analysis.
</commit_message>
<xml_diff>
--- a/demo/demo4-complete/output/post-method-series.xlsx
+++ b/demo/demo4-complete/output/post-method-series.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnostics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Diagnostics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -139,7 +139,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>

</xml_diff>